<commit_message>
Added source, column name descriptions, photos and other metadata
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedDigestibility.xlsx
+++ b/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedDigestibility.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Verson control in Git\ApsimX\Tests\Validation\System\NarayenLongTermGrazingTrial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FF6A8A-93C0-4B9B-A744-962400CFF925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF21C449-228F-4495-8D39-AA54185A28A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57390" yWindow="0" windowWidth="19410" windowHeight="20880" xr2:uid="{1A988655-30E2-4E9A-8043-C550654892FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{1A988655-30E2-4E9A-8043-C550654892FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Observed" sheetId="1" r:id="rId1"/>
+    <sheet name="Tech memo appendix e" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="29">
   <si>
     <t>SimulationName</t>
   </si>
@@ -83,6 +84,30 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>nitrogen</t>
+  </si>
+  <si>
+    <t>pasture_type</t>
+  </si>
+  <si>
+    <t>green_panic</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>rhodes_grass</t>
+  </si>
+  <si>
+    <t>unsown_grasses</t>
+  </si>
+  <si>
+    <t>Tech memo appendix E digitised by Julian Rich</t>
   </si>
 </sst>
 </file>
@@ -3120,4 +3145,1034 @@
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46F9880-A7D8-49DC-A3F6-4461998E25F0}">
+  <dimension ref="A1:L39"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>1.4</v>
+      </c>
+      <c r="D1">
+        <v>1.8</v>
+      </c>
+      <c r="E1">
+        <v>2</v>
+      </c>
+      <c r="F1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>26842</v>
+      </c>
+      <c r="B2">
+        <v>60.5</v>
+      </c>
+      <c r="C2">
+        <v>64.5</v>
+      </c>
+      <c r="D2">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="E2">
+        <v>65.7</v>
+      </c>
+      <c r="F2">
+        <v>57</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>26981</v>
+      </c>
+      <c r="B3">
+        <v>59.5</v>
+      </c>
+      <c r="C3">
+        <v>66</v>
+      </c>
+      <c r="D3">
+        <v>65.8</v>
+      </c>
+      <c r="E3">
+        <v>65.7</v>
+      </c>
+      <c r="F3">
+        <v>67</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>27046</v>
+      </c>
+      <c r="B4">
+        <v>58.8</v>
+      </c>
+      <c r="C4">
+        <v>57.7</v>
+      </c>
+      <c r="D4">
+        <v>53.2</v>
+      </c>
+      <c r="E4">
+        <v>54.2</v>
+      </c>
+      <c r="F4">
+        <v>56.6</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>27092</v>
+      </c>
+      <c r="B5">
+        <v>52.3</v>
+      </c>
+      <c r="C5">
+        <v>53.3</v>
+      </c>
+      <c r="D5">
+        <v>53.9</v>
+      </c>
+      <c r="E5">
+        <v>54.7</v>
+      </c>
+      <c r="F5">
+        <v>51</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>27149</v>
+      </c>
+      <c r="B6">
+        <v>48.1</v>
+      </c>
+      <c r="C6">
+        <v>49.1</v>
+      </c>
+      <c r="D6">
+        <v>47.7</v>
+      </c>
+      <c r="E6">
+        <v>47.5</v>
+      </c>
+      <c r="F6">
+        <v>51</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>27204</v>
+      </c>
+      <c r="B7">
+        <v>41.8</v>
+      </c>
+      <c r="C7">
+        <v>41.3</v>
+      </c>
+      <c r="D7">
+        <v>37.700000000000003</v>
+      </c>
+      <c r="E7">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="F7">
+        <v>44.3</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>27261</v>
+      </c>
+      <c r="B8">
+        <v>44.8</v>
+      </c>
+      <c r="C8">
+        <v>44.8</v>
+      </c>
+      <c r="D8">
+        <v>40.4</v>
+      </c>
+      <c r="E8">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="F8">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>27325</v>
+      </c>
+      <c r="B9">
+        <v>67.099999999999994</v>
+      </c>
+      <c r="C9">
+        <v>66.599999999999994</v>
+      </c>
+      <c r="D9">
+        <v>64.400000000000006</v>
+      </c>
+      <c r="E9">
+        <v>65.3</v>
+      </c>
+      <c r="F9">
+        <v>67</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B10">
+        <v>61</v>
+      </c>
+      <c r="C10">
+        <v>60.7</v>
+      </c>
+      <c r="D10">
+        <v>62.4</v>
+      </c>
+      <c r="E10">
+        <v>57.8</v>
+      </c>
+      <c r="F10">
+        <v>64</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B11">
+        <v>50.7</v>
+      </c>
+      <c r="C11">
+        <v>49.7</v>
+      </c>
+      <c r="D11">
+        <v>53</v>
+      </c>
+      <c r="E11">
+        <v>53.7</v>
+      </c>
+      <c r="F11">
+        <v>47.3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>27485</v>
+      </c>
+      <c r="B12">
+        <v>53.7</v>
+      </c>
+      <c r="C12">
+        <v>58.3</v>
+      </c>
+      <c r="D12">
+        <v>57.3</v>
+      </c>
+      <c r="E12">
+        <v>60.3</v>
+      </c>
+      <c r="F12">
+        <v>61.3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B13">
+        <v>37.6</v>
+      </c>
+      <c r="C13">
+        <v>41.7</v>
+      </c>
+      <c r="D13">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="E13">
+        <v>38.4</v>
+      </c>
+      <c r="F13">
+        <v>39.4</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>26842</v>
+      </c>
+      <c r="B14">
+        <v>61.9</v>
+      </c>
+      <c r="C14">
+        <v>63.9</v>
+      </c>
+      <c r="D14">
+        <v>65.3</v>
+      </c>
+      <c r="E14">
+        <v>63</v>
+      </c>
+      <c r="F14">
+        <v>66.400000000000006</v>
+      </c>
+      <c r="G14">
+        <v>100</v>
+      </c>
+      <c r="H14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>26981</v>
+      </c>
+      <c r="B15">
+        <v>69.7</v>
+      </c>
+      <c r="C15">
+        <v>67.900000000000006</v>
+      </c>
+      <c r="D15">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="E15">
+        <v>72.900000000000006</v>
+      </c>
+      <c r="F15">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="G15">
+        <v>100</v>
+      </c>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>27046</v>
+      </c>
+      <c r="B16">
+        <v>54.3</v>
+      </c>
+      <c r="C16">
+        <v>56.6</v>
+      </c>
+      <c r="D16">
+        <v>52.8</v>
+      </c>
+      <c r="E16">
+        <v>55.8</v>
+      </c>
+      <c r="F16">
+        <v>55.9</v>
+      </c>
+      <c r="G16">
+        <v>100</v>
+      </c>
+      <c r="H16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>27092</v>
+      </c>
+      <c r="B17">
+        <v>52.7</v>
+      </c>
+      <c r="C17">
+        <v>56.5</v>
+      </c>
+      <c r="D17">
+        <v>53.3</v>
+      </c>
+      <c r="E17">
+        <v>55.1</v>
+      </c>
+      <c r="F17">
+        <v>51.8</v>
+      </c>
+      <c r="G17">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>27149</v>
+      </c>
+      <c r="B18">
+        <v>50.2</v>
+      </c>
+      <c r="C18">
+        <v>49.4</v>
+      </c>
+      <c r="D18">
+        <v>52.8</v>
+      </c>
+      <c r="E18">
+        <v>52.5</v>
+      </c>
+      <c r="F18">
+        <v>50.3</v>
+      </c>
+      <c r="G18">
+        <v>100</v>
+      </c>
+      <c r="H18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>27204</v>
+      </c>
+      <c r="B19">
+        <v>42.4</v>
+      </c>
+      <c r="C19">
+        <v>37.4</v>
+      </c>
+      <c r="D19">
+        <v>35.5</v>
+      </c>
+      <c r="E19">
+        <v>39.4</v>
+      </c>
+      <c r="F19">
+        <v>36.5</v>
+      </c>
+      <c r="G19">
+        <v>100</v>
+      </c>
+      <c r="H19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>27261</v>
+      </c>
+      <c r="B20">
+        <v>42.3</v>
+      </c>
+      <c r="C20">
+        <v>39.200000000000003</v>
+      </c>
+      <c r="D20">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="E20">
+        <v>40.6</v>
+      </c>
+      <c r="F20">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="G20">
+        <v>100</v>
+      </c>
+      <c r="H20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>27325</v>
+      </c>
+      <c r="B21">
+        <v>67.900000000000006</v>
+      </c>
+      <c r="C21">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="D21">
+        <v>70.3</v>
+      </c>
+      <c r="E21">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="F21">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="G21">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B22">
+        <v>63.4</v>
+      </c>
+      <c r="C22">
+        <v>63</v>
+      </c>
+      <c r="D22">
+        <v>62</v>
+      </c>
+      <c r="E22">
+        <v>61.5</v>
+      </c>
+      <c r="F22">
+        <v>62.2</v>
+      </c>
+      <c r="G22">
+        <v>100</v>
+      </c>
+      <c r="H22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B23">
+        <v>50</v>
+      </c>
+      <c r="C23">
+        <v>46.5</v>
+      </c>
+      <c r="D23">
+        <v>49.8</v>
+      </c>
+      <c r="E23">
+        <v>53</v>
+      </c>
+      <c r="F23">
+        <v>50.8</v>
+      </c>
+      <c r="G23">
+        <v>100</v>
+      </c>
+      <c r="H23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>27485</v>
+      </c>
+      <c r="B24">
+        <v>54.5</v>
+      </c>
+      <c r="C24">
+        <v>54.4</v>
+      </c>
+      <c r="D24">
+        <v>57.7</v>
+      </c>
+      <c r="E24">
+        <v>58.3</v>
+      </c>
+      <c r="F24">
+        <v>55.3</v>
+      </c>
+      <c r="G24">
+        <v>100</v>
+      </c>
+      <c r="H24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B25">
+        <v>40.5</v>
+      </c>
+      <c r="C25">
+        <v>39.9</v>
+      </c>
+      <c r="D25">
+        <v>40.4</v>
+      </c>
+      <c r="E25">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="F25">
+        <v>43.3</v>
+      </c>
+      <c r="G25">
+        <v>100</v>
+      </c>
+      <c r="H25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26">
+        <v>55.3</v>
+      </c>
+      <c r="D26" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26">
+        <v>54.1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B27">
+        <v>44</v>
+      </c>
+      <c r="C27">
+        <v>47.7</v>
+      </c>
+      <c r="D27">
+        <v>48.2</v>
+      </c>
+      <c r="E27">
+        <v>44.9</v>
+      </c>
+      <c r="F27">
+        <v>51.4</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>27485</v>
+      </c>
+      <c r="B28">
+        <v>51.5</v>
+      </c>
+      <c r="C28">
+        <v>53.8</v>
+      </c>
+      <c r="D28">
+        <v>56.5</v>
+      </c>
+      <c r="E28">
+        <v>55.2</v>
+      </c>
+      <c r="F28">
+        <v>52.1</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29">
+        <v>36.5</v>
+      </c>
+      <c r="D29">
+        <v>39.6</v>
+      </c>
+      <c r="E29">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="F29">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B30">
+        <v>54.5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30">
+        <v>53.8</v>
+      </c>
+      <c r="F30">
+        <v>57.7</v>
+      </c>
+      <c r="G30">
+        <v>100</v>
+      </c>
+      <c r="H30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B31">
+        <v>44.2</v>
+      </c>
+      <c r="C31">
+        <v>48.7</v>
+      </c>
+      <c r="D31">
+        <v>42.6</v>
+      </c>
+      <c r="E31">
+        <v>39.5</v>
+      </c>
+      <c r="F31">
+        <v>47.6</v>
+      </c>
+      <c r="G31">
+        <v>100</v>
+      </c>
+      <c r="H31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>27485</v>
+      </c>
+      <c r="B32">
+        <v>47.9</v>
+      </c>
+      <c r="C32">
+        <v>53.7</v>
+      </c>
+      <c r="D32">
+        <v>51</v>
+      </c>
+      <c r="E32">
+        <v>55.1</v>
+      </c>
+      <c r="F32">
+        <v>52</v>
+      </c>
+      <c r="G32">
+        <v>100</v>
+      </c>
+      <c r="H32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B33">
+        <v>31</v>
+      </c>
+      <c r="C33">
+        <v>29.5</v>
+      </c>
+      <c r="D33">
+        <v>35</v>
+      </c>
+      <c r="E33">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F33">
+        <v>29.6</v>
+      </c>
+      <c r="G33">
+        <v>100</v>
+      </c>
+      <c r="H33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34">
+        <v>54.5</v>
+      </c>
+      <c r="D34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35">
+        <v>48.1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B36" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36">
+        <v>44.3</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>27382</v>
+      </c>
+      <c r="B37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" t="s">
+        <v>25</v>
+      </c>
+      <c r="E37" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37">
+        <v>100</v>
+      </c>
+      <c r="H37" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>27429</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" t="s">
+        <v>25</v>
+      </c>
+      <c r="E38" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38">
+        <v>100</v>
+      </c>
+      <c r="H38" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>27541</v>
+      </c>
+      <c r="B39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39">
+        <v>100</v>
+      </c>
+      <c r="H39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Created Observed OM spreadsheet, add info to the metadata of the others
Created Observed OM spreadsheet, add info to the metadata of the others
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedDigestibility.xlsx
+++ b/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedDigestibility.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Verson control in Git\ApsimX\Tests\Validation\System\NarayenLongTermGrazingTrial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF21C449-228F-4495-8D39-AA54185A28A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A8BB73-A91A-494F-BA33-2C1F28771BC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{1A988655-30E2-4E9A-8043-C550654892FB}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{1A988655-30E2-4E9A-8043-C550654892FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Observed" sheetId="1" r:id="rId1"/>
@@ -652,6 +652,55 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>48823</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>30254</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9143A308-2FC8-4C7B-B2C9-D6508DDA88B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5959929" y="370114"/>
+          <a:ext cx="9192823" cy="11688854"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -970,13 +1019,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A677579D-2008-4422-89BD-2B9140BD879F}">
   <dimension ref="A1:F121"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="5" max="5" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -996,7 +1045,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1013,7 +1062,7 @@
         <v>60.5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1030,7 +1079,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1047,7 +1096,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1064,7 +1113,7 @@
         <v>52.3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1081,7 +1130,7 @@
         <v>48.1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1098,7 +1147,7 @@
         <v>41.8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1115,7 +1164,7 @@
         <v>44.8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1132,7 +1181,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1149,7 +1198,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1169,7 +1218,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1189,7 +1238,7 @@
         <v>51.5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1206,7 +1255,7 @@
         <v>37.6</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -1223,7 +1272,7 @@
         <v>61.9</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1240,7 +1289,7 @@
         <v>69.7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -1257,7 +1306,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -1274,7 +1323,7 @@
         <v>52.7</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -1291,7 +1340,7 @@
         <v>50.2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -1308,7 +1357,7 @@
         <v>42.4</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -1325,7 +1374,7 @@
         <v>42.3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -1342,7 +1391,7 @@
         <v>67.900000000000006</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -1362,7 +1411,7 @@
         <v>54.5</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -1382,7 +1431,7 @@
         <v>44.2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -1402,7 +1451,7 @@
         <v>47.9</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>7</v>
       </c>
@@ -1422,7 +1471,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1439,7 +1488,7 @@
         <v>64.5</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1456,7 +1505,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1473,7 +1522,7 @@
         <v>57.7</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1490,7 +1539,7 @@
         <v>53.3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1507,7 +1556,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1524,7 +1573,7 @@
         <v>41.3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1541,7 +1590,7 @@
         <v>44.8</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1558,7 +1607,7 @@
         <v>66.599999999999994</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1578,7 +1627,7 @@
         <v>55.3</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1598,7 +1647,7 @@
         <v>47.7</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1618,7 +1667,7 @@
         <v>53.8</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1638,7 +1687,7 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -1655,7 +1704,7 @@
         <v>63.9</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>10</v>
       </c>
@@ -1672,7 +1721,7 @@
         <v>67.900000000000006</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>10</v>
       </c>
@@ -1689,7 +1738,7 @@
         <v>56.6</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>10</v>
       </c>
@@ -1706,7 +1755,7 @@
         <v>56.5</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>10</v>
       </c>
@@ -1723,7 +1772,7 @@
         <v>49.4</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -1740,7 +1789,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>10</v>
       </c>
@@ -1757,7 +1806,7 @@
         <v>39.200000000000003</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>10</v>
       </c>
@@ -1774,7 +1823,7 @@
         <v>67.599999999999994</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>10</v>
       </c>
@@ -1791,7 +1840,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>10</v>
       </c>
@@ -1811,7 +1860,7 @@
         <v>48.7</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>10</v>
       </c>
@@ -1831,7 +1880,7 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>10</v>
       </c>
@@ -1851,7 +1900,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>11</v>
       </c>
@@ -1868,7 +1917,7 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -1885,7 +1934,7 @@
         <v>65.8</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>11</v>
       </c>
@@ -1902,7 +1951,7 @@
         <v>53.2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>11</v>
       </c>
@@ -1919,7 +1968,7 @@
         <v>53.9</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>11</v>
       </c>
@@ -1936,7 +1985,7 @@
         <v>47.7</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>11</v>
       </c>
@@ -1953,7 +2002,7 @@
         <v>37.700000000000003</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>11</v>
       </c>
@@ -1970,7 +2019,7 @@
         <v>40.4</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>11</v>
       </c>
@@ -1987,7 +2036,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>11</v>
       </c>
@@ -2004,7 +2053,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>11</v>
       </c>
@@ -2024,7 +2073,7 @@
         <v>48.2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>11</v>
       </c>
@@ -2044,7 +2093,7 @@
         <v>56.5</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>11</v>
       </c>
@@ -2064,7 +2113,7 @@
         <v>39.6</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>13</v>
       </c>
@@ -2081,7 +2130,7 @@
         <v>65.3</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -2098,7 +2147,7 @@
         <v>71.400000000000006</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -2115,7 +2164,7 @@
         <v>52.8</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -2132,7 +2181,7 @@
         <v>53.3</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -2149,7 +2198,7 @@
         <v>52.8</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -2166,7 +2215,7 @@
         <v>35.5</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -2183,7 +2232,7 @@
         <v>37.799999999999997</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -2200,7 +2249,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -2217,7 +2266,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -2237,7 +2286,7 @@
         <v>42.6</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -2257,7 +2306,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -2277,7 +2326,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -2294,7 +2343,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>14</v>
       </c>
@@ -2311,7 +2360,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -2328,7 +2377,7 @@
         <v>54.2</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>14</v>
       </c>
@@ -2345,7 +2394,7 @@
         <v>54.7</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -2362,7 +2411,7 @@
         <v>47.5</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>14</v>
       </c>
@@ -2379,7 +2428,7 @@
         <v>38.700000000000003</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>14</v>
       </c>
@@ -2396,7 +2445,7 @@
         <v>38.299999999999997</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>14</v>
       </c>
@@ -2413,7 +2462,7 @@
         <v>65.3</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>14</v>
       </c>
@@ -2433,7 +2482,7 @@
         <v>54.1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>14</v>
       </c>
@@ -2453,7 +2502,7 @@
         <v>44.9</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -2473,7 +2522,7 @@
         <v>55.2</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>14</v>
       </c>
@@ -2493,7 +2542,7 @@
         <v>38.799999999999997</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -2510,7 +2559,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>16</v>
       </c>
@@ -2527,7 +2576,7 @@
         <v>72.900000000000006</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>16</v>
       </c>
@@ -2544,7 +2593,7 @@
         <v>55.8</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>16</v>
       </c>
@@ -2561,7 +2610,7 @@
         <v>55.1</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>16</v>
       </c>
@@ -2578,7 +2627,7 @@
         <v>52.5</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>16</v>
       </c>
@@ -2595,7 +2644,7 @@
         <v>39.4</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>16</v>
       </c>
@@ -2612,7 +2661,7 @@
         <v>40.6</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>16</v>
       </c>
@@ -2629,7 +2678,7 @@
         <v>67.599999999999994</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>16</v>
       </c>
@@ -2649,7 +2698,7 @@
         <v>53.8</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>16</v>
       </c>
@@ -2669,7 +2718,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>16</v>
       </c>
@@ -2689,7 +2738,7 @@
         <v>55.1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>16</v>
       </c>
@@ -2709,7 +2758,7 @@
         <v>32.799999999999997</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>17</v>
       </c>
@@ -2726,7 +2775,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>17</v>
       </c>
@@ -2743,7 +2792,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>17</v>
       </c>
@@ -2760,7 +2809,7 @@
         <v>56.6</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>17</v>
       </c>
@@ -2777,7 +2826,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
         <v>17</v>
       </c>
@@ -2794,7 +2843,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>17</v>
       </c>
@@ -2811,7 +2860,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>17</v>
       </c>
@@ -2828,7 +2877,7 @@
         <v>38.700000000000003</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
         <v>17</v>
       </c>
@@ -2845,7 +2894,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
         <v>17</v>
       </c>
@@ -2862,7 +2911,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>17</v>
       </c>
@@ -2882,7 +2931,7 @@
         <v>51.4</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>17</v>
       </c>
@@ -2902,7 +2951,7 @@
         <v>52.1</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
         <v>17</v>
       </c>
@@ -2922,7 +2971,7 @@
         <v>34.299999999999997</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
         <v>19</v>
       </c>
@@ -2939,7 +2988,7 @@
         <v>66.400000000000006</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
         <v>19</v>
       </c>
@@ -2956,7 +3005,7 @@
         <v>71.099999999999994</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>19</v>
       </c>
@@ -2973,7 +3022,7 @@
         <v>55.9</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>19</v>
       </c>
@@ -2990,7 +3039,7 @@
         <v>51.8</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>19</v>
       </c>
@@ -3007,7 +3056,7 @@
         <v>50.3</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>19</v>
       </c>
@@ -3024,7 +3073,7 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>19</v>
       </c>
@@ -3041,7 +3090,7 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
         <v>19</v>
       </c>
@@ -3058,7 +3107,7 @@
         <v>70.099999999999994</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
         <v>19</v>
       </c>
@@ -3078,7 +3127,7 @@
         <v>57.7</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
         <v>19</v>
       </c>
@@ -3098,7 +3147,7 @@
         <v>47.6</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
         <v>19</v>
       </c>
@@ -3118,7 +3167,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
         <v>19</v>
       </c>
@@ -3150,12 +3199,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46F9880-A7D8-49DC-A3F6-4461998E25F0}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -3184,7 +3233,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>26842</v>
       </c>
@@ -3210,7 +3259,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>26981</v>
       </c>
@@ -3236,7 +3285,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>27046</v>
       </c>
@@ -3262,7 +3311,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>27092</v>
       </c>
@@ -3288,7 +3337,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>27149</v>
       </c>
@@ -3314,7 +3363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>27204</v>
       </c>
@@ -3340,7 +3389,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>27261</v>
       </c>
@@ -3366,7 +3415,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>27325</v>
       </c>
@@ -3392,7 +3441,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>27382</v>
       </c>
@@ -3418,7 +3467,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>27429</v>
       </c>
@@ -3444,7 +3493,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>27485</v>
       </c>
@@ -3470,7 +3519,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>27541</v>
       </c>
@@ -3496,7 +3545,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>26842</v>
       </c>
@@ -3522,7 +3571,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>26981</v>
       </c>
@@ -3548,7 +3597,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>27046</v>
       </c>
@@ -3574,7 +3623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>27092</v>
       </c>
@@ -3600,7 +3649,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>27149</v>
       </c>
@@ -3626,7 +3675,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>27204</v>
       </c>
@@ -3652,7 +3701,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>27261</v>
       </c>
@@ -3678,7 +3727,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>27325</v>
       </c>
@@ -3704,7 +3753,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>27382</v>
       </c>
@@ -3730,7 +3779,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>27429</v>
       </c>
@@ -3756,7 +3805,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>27485</v>
       </c>
@@ -3782,7 +3831,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>27541</v>
       </c>
@@ -3808,7 +3857,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>27382</v>
       </c>
@@ -3834,7 +3883,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27" s="1">
         <v>27429</v>
       </c>
@@ -3860,7 +3909,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A28" s="1">
         <v>27485</v>
       </c>
@@ -3886,7 +3935,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29" s="1">
         <v>27541</v>
       </c>
@@ -3912,7 +3961,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30" s="1">
         <v>27382</v>
       </c>
@@ -3938,7 +3987,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A31" s="1">
         <v>27429</v>
       </c>
@@ -3964,7 +4013,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A32" s="1">
         <v>27485</v>
       </c>
@@ -3990,7 +4039,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33" s="1">
         <v>27541</v>
       </c>
@@ -4016,7 +4065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A34" s="1">
         <v>27382</v>
       </c>
@@ -4042,7 +4091,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35" s="1">
         <v>27429</v>
       </c>
@@ -4068,7 +4117,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36" s="1">
         <v>27541</v>
       </c>
@@ -4094,7 +4143,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A37" s="1">
         <v>27382</v>
       </c>
@@ -4120,7 +4169,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A38" s="1">
         <v>27429</v>
       </c>
@@ -4146,7 +4195,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39" s="1">
         <v>27541</v>
       </c>
@@ -4174,5 +4223,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>